<commit_message>
Modifies url changes and fixed few issues
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/isa-open-valid.xlsx
+++ b/src/test/resources/testData/isa-open-valid.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vinay.Varghese/disa-returns-frontend-ui-tests/src/test/resources/testData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/divya.natarajan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91802329-C0B9-7C4A-9AA8-E16F87B3B0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42AA5A3E-EC21-0A4B-9725-18637593736E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly return" sheetId="1" r:id="rId1"/>
@@ -126,7 +126,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -156,7 +156,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -596,7 +596,7 @@
         <v>30</v>
       </c>
       <c r="L3" s="1">
-        <v>46242</v>
+        <v>46211</v>
       </c>
       <c r="M3" t="s">
         <v>31</v>

</xml_diff>